<commit_message>
Add duplicate and validation logic
</commit_message>
<xml_diff>
--- a/job_applications.xlsx
+++ b/job_applications.xlsx
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:I21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>company</v>
+        <v>Company</v>
       </c>
       <c r="B1" t="str">
         <v>Role</v>
@@ -417,6 +417,15 @@
       </c>
       <c r="F1" t="str">
         <v>Work_mode</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Job_id</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Applied</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Referral_asked</v>
       </c>
     </row>
     <row r="2">
@@ -427,21 +436,572 @@
         <v>ABC</v>
       </c>
       <c r="C2" t="str">
+        <v>09</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Anywhere</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Nothing</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Anywhere</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="D3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="G3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="H3" t="str">
+        <v>New1</v>
+      </c>
+      <c r="I3" t="str">
+        <v>New1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>New1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>New2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>New1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>New1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>New1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>New1</v>
+      </c>
+      <c r="G4" t="str">
+        <v>New2</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I4" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Enter job role: New2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Enter experience required:New1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Enter location: New1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Enter required skills: New1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Enter work mode: New1</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Enter job ID: New2</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Have you applied? Yes/No: Yes</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Asked for referral? Yes/No: No</v>
+      </c>
+      <c r="I5" t="str">
+        <v>asdad</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>New1</v>
+      </c>
+      <c r="B6" t="str">
+        <v>New2</v>
+      </c>
+      <c r="C6" t="str">
+        <v>New1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>New1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>New1</v>
+      </c>
+      <c r="F6" t="str">
+        <v>New1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>New3</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I6" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B7" t="str">
+        <v>New1</v>
+      </c>
+      <c r="C7" t="str">
         <v>02</v>
       </c>
-      <c r="D2" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="E2" t="str">
-        <v>ABC</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Remote</v>
+      <c r="D7" t="str">
+        <v>New1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Nothing</v>
+      </c>
+      <c r="F7" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G7" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H7" t="str">
+        <v>yes</v>
+      </c>
+      <c r="I7" t="str">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B8" t="str">
+        <v>New1</v>
+      </c>
+      <c r="C8" t="str">
+        <v>02</v>
+      </c>
+      <c r="D8" t="str">
+        <v>New1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Nothing</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Nothing</v>
+      </c>
+      <c r="G8" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I8" t="str">
+        <v>no</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Role1</v>
+      </c>
+      <c r="C9" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D9" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E9" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F9" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G9" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H9" t="str">
+        <v>YEs</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Role1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D10" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E10" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F10" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G10" t="str">
+        <v>ID02</v>
+      </c>
+      <c r="H10" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I10" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>comp1</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Role2</v>
+      </c>
+      <c r="C11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G11" t="str">
+        <v>ID03</v>
+      </c>
+      <c r="H11" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I11" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Comp2</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Role1</v>
+      </c>
+      <c r="C12" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D12" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E12" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F12" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G12" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H12" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I12" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Role4</v>
+      </c>
+      <c r="C13" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D13" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E13" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F13" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G13" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H13" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I13" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Role1</v>
+      </c>
+      <c r="C14" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D14" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E14" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F14" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G14" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H14" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I14" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Comp1</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Role1</v>
+      </c>
+      <c r="C15" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D15" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E15" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F15" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G15" t="str">
+        <v>ID01</v>
+      </c>
+      <c r="H15" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I15" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>comp1</v>
+      </c>
+      <c r="B16" t="str">
+        <v>role7</v>
+      </c>
+      <c r="C16" t="str">
+        <v>03</v>
+      </c>
+      <c r="D16" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E16" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F16" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G16" t="str">
+        <v>ID09</v>
+      </c>
+      <c r="H16" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I16" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Comp4</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Role3</v>
+      </c>
+      <c r="C17" t="str">
+        <v>NA</v>
+      </c>
+      <c r="D17" t="str">
+        <v>NA</v>
+      </c>
+      <c r="E17" t="str">
+        <v>NA</v>
+      </c>
+      <c r="F17" t="str">
+        <v>NA</v>
+      </c>
+      <c r="G17" t="str">
+        <v>ID09</v>
+      </c>
+      <c r="H17" t="str">
+        <v>NA</v>
+      </c>
+      <c r="I17" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>COMP12</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Role12</v>
+      </c>
+      <c r="C18" t="str">
+        <v>na</v>
+      </c>
+      <c r="D18" t="str">
+        <v>na</v>
+      </c>
+      <c r="E18" t="str">
+        <v>na</v>
+      </c>
+      <c r="F18" t="str">
+        <v>na</v>
+      </c>
+      <c r="G18" t="str">
+        <v>ID12</v>
+      </c>
+      <c r="H18" t="str">
+        <v>na</v>
+      </c>
+      <c r="I18" t="str">
+        <v>na</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>comp12</v>
+      </c>
+      <c r="B20" t="str">
+        <v>rol45</v>
+      </c>
+      <c r="C20" t="str">
+        <v>na</v>
+      </c>
+      <c r="D20" t="str">
+        <v>na</v>
+      </c>
+      <c r="E20" t="str">
+        <v>na</v>
+      </c>
+      <c r="F20" t="str">
+        <v>na</v>
+      </c>
+      <c r="G20" t="str">
+        <v>id45</v>
+      </c>
+      <c r="H20" t="str">
+        <v>na</v>
+      </c>
+      <c r="I20" t="str">
+        <v>na</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>comp-1</v>
+      </c>
+      <c r="B21" t="str">
+        <v>ROLE_2</v>
+      </c>
+      <c r="C21" t="str">
+        <v>10-12</v>
+      </c>
+      <c r="D21" t="str">
+        <v>*Only in Asia</v>
+      </c>
+      <c r="E21" t="str">
+        <v>SQL &amp; Manual testing</v>
+      </c>
+      <c r="F21" t="str">
+        <v>100% Remote</v>
+      </c>
+      <c r="G21" t="str">
+        <v>ID23</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Nope</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Never</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>